<commit_message>
Render PDF tiles across CPU cores with shared pixel buffers
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R2606efef7ad94685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Rbc1317c6ff0f4c3b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1190,10 +1190,10 @@
         <x:v>99</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="45" customHeight="1">
+    <x:row r="105" ht="72" customHeight="1">
       <x:c r="A105"/>
       <x:c r="B105" s="4" t="str">
-        <x:v>Improve responsiveness and reliability when opening, scrolling, zooming and editing PDFs; measure performance on dense drawings and repair reproducible stalls or interaction failures.</x:v>
+        <x:v>Improve responsiveness and reliability when opening, scrolling, zooming and editing PDFs. Use multiple CPU cores safely for background rendering, retain reusable parsed pages, prioritise visible tiles and cancel obsolete work. Measure dense-drawing rendering speed and UI responsiveness without reducing image quality or allowing unbounded memory use.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Recover Escape across focus and mouse grabs and verify remaining tasks
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Rbc1317c6ff0f4c3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R6a96d17eefb04d33"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -613,10 +613,10 @@
         <x:v>4</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="56" customHeight="1">
+    <x:row r="6" ht="72" customHeight="1">
       <x:c r="A6" s="2"/>
       <x:c r="B6" s="3" t="str">
-        <x:v>Fix tool states that prevent cancellation or switching tools, including after placing a callout arrow. Abandon stale callout anchors and held toolset payloads when changing tools. A callout-switching defect was reproduced and repaired on 2026-09-12; the reported Escape-resistant lockup still needs a reproducing sequence (82, 110)</x:v>
+        <x:v>Fix tool states that prevent cancellation or switching tools, including after placing a callout arrow. Abandon stale callout anchors and held toolset payloads when changing tools. Callout switching, Escape swallowed by inline panel editors, and stale scene mouse grabs have reproduced fixes and Qt regression coverage. Confirmation against the original reported sequence remains pending (82, 110)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="90">

</xml_diff>

<commit_message>
Speed up editing and undo by removing repeated UI work
Page restoration rebuilt the panels for every removed markup, making undo quadratic. Publish one completed page change, reuse serialized undo state and nearby snap candidates, and avoid repeated style traversal, unit parsing and widget ownership checks. Preserve full document state and interaction behavior, with native before/after benchmarks, 920 passing tests and a 1000-round stress run.
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R6a96d17eefb04d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R93c14452591543e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1190,10 +1190,10 @@
         <x:v>99</x:v>
       </x:c>
     </x:row>
-    <x:row r="105" ht="72" customHeight="1">
+    <x:row r="105" ht="90" customHeight="1">
       <x:c r="A105"/>
       <x:c r="B105" s="4" t="str">
-        <x:v>Improve responsiveness and reliability when opening, scrolling, zooming and editing PDFs. Use multiple CPU cores safely for background rendering, retain reusable parsed pages, prioritise visible tiles and cancel obsolete work. Measure dense-drawing rendering speed and UI responsiveness without reducing image quality or allowing unbounded memory use.</x:v>
+        <x:v>Make the application as fast and responsive as practical without compromising functionality, usability or visual quality. Profile opening, scrolling, zooming, snapping, editing and undo on demanding documents. Use multiple CPU cores safely for background PDF rendering, retain reusable parsed pages, prioritise visible tiles and cancel obsolete work. Remove redundant work, measure improvements and keep memory bounded.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="45" customHeight="1">

</xml_diff>

<commit_message>
Repair PDF export, snapping, and markup style controls
Export painted viewing paper into PDFs and Save omitted contents links, while PDF vectors were unavailable to snapping. Remove the paper paint, write links on both save paths, and query source vector geometry without turning it into markups.

Add a temporary calibration guide, reliable second-point and curve previews, shared view synchronization, editable break symbols, numeric style controls and visual line endings. Save atomically while retaining Undo assets. Record the reported requirements and remaining acceptance checks, and validate with the full suite and native stress session.
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="R93c14452591543e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Rd77c7659314b4c28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -340,7 +340,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="top"/>
@@ -353,6 +353,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1262,8 +1265,104 @@
         <x:v>(found during 2026-09-11 walkthrough) Section header/footer columns must remain readable and editable in the default dialog width; Insert PDF preview instructions must wrap within the preview.</x:v>
       </x:c>
     </x:row>
+    <x:row r="117" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A117" s="5"/>
+      <x:c r="B117" s="5" t="str">
+        <x:v>Exported PDFs must not introduce an opaque white page background that appears when taking a snapshot in Bluebeam. Verify actual PDF content and transparency in saved/exported output.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="15" hidden="0" customHeight="1">
+      <x:c r="A118" s="5"/>
+      <x:c r="B118" s="5" t="str">
+        <x:v>Two-point scale calibration must show only a temporary dashed guide with a consistent on-screen size, without dimension graphics or a permanent measurement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A119" s="5"/>
+      <x:c r="B119" s="5" t="str">
+        <x:v>Replace sliders with editable numeric controls and visible up/down buttons for opacity, font size, thickness and other numeric styles in both Properties and the style toolbar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="15" hidden="0" customHeight="1">
+      <x:c r="A120" s="5"/>
+      <x:c r="B120" s="5" t="str">
+        <x:v>Arrowheads must finish at a sharp point. Show visual arrowhead previews in line-end dropdowns and the style toolbar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A121" s="5"/>
+      <x:c r="B121" s="5" t="str">
+        <x:v>Title-block hyperlinks must work in exported PDFs opened in other viewers. Support selected paper size with a chosen quantity or fit option; clarify whether the quantity refers to pages or title blocks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A122" s="5"/>
+      <x:c r="B122" s="5" t="str">
+        <x:v>Changing view synchronization must apply across all windows and split views of the same document, without enabling it separately in each view. Repair zoom and cursor anchoring while Document sync is active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="15" hidden="0" customHeight="1">
+      <x:c r="A123" s="5"/>
+      <x:c r="B123" s="5" t="str">
+        <x:v>Live polygon/segment curve edits must not clip when the preview extends beyond its previous bounds or viewport; update the preview throughout the gesture.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124" ht="15" hidden="0" customHeight="1">
+      <x:c r="A124" s="5"/>
+      <x:c r="B124" s="5" t="str">
+        <x:v>Snapshot outline defaults must persist and apply to subsequent snapshots.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125" ht="15" hidden="0" customHeight="1">
+      <x:c r="A125" s="5"/>
+      <x:c r="B125" s="5" t="str">
+        <x:v>Structural break lines must expose size and placement controls, including moving the break along its segment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="15" hidden="0" customHeight="1">
+      <x:c r="A126" s="5"/>
+      <x:c r="B126" s="5" t="str">
+        <x:v>Repair alignment snapping during second-point placement; guides and snapped geometry must remain stable and agree.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="15" hidden="0" customHeight="1">
+      <x:c r="A127" s="5"/>
+      <x:c r="B127" s="5" t="str">
+        <x:v>Repair snapping to PDF content, including endpoints and intersections.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="15" hidden="0" customHeight="1">
+      <x:c r="A128" s="5"/>
+      <x:c r="B128" s="5" t="str">
+        <x:v>Clarify the unfinished report “whiteout should”; retain existing Whiteout requirements pending the missing detail.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A129" s="5"/>
+      <x:c r="B129" s="5" t="str">
+        <x:v>Fix excessive window minimum width on Windows: a 1920-pixel display currently requests a 1941-pixel client width and triggers QWindowsWindow::setGeometry warnings. Controls must remain accessible at that display size.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A130" s="5"/>
+      <x:c r="B130" s="5" t="str">
+        <x:v>Run the full automated suite and a fresh visual mouse/keyboard walkthrough of existing features; compare Bluebeam terminology, colours, formatting and workflows. Record concrete issues and repair them.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A131" s="5"/>
+      <x:c r="B131" s="5" t="str">
+        <x:v>Audit every markup type: expose all applicable editable properties in Properties, and important colour, hatch, line-end, arrowhead, line-style, thickness and opacity controls in the style toolbar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="15" hidden="0" customHeight="1">
+      <x:c r="A132" s="5"/>
+      <x:c r="B132" s="5" t="str">
+        <x:v>Continue profiling and improving responsiveness without reducing rendering quality or functionality, including synchronized zoom, drawing previews and snapping.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:B116"/>
+  <x:autoFilter ref="A1:B132"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix PDF snapping guides and break controls
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Rd77c7659314b4c28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task list" sheetId="1" r:id="Rdc96bbb66d1c4662"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1292,7 +1292,7 @@
     <x:row r="121" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A121" s="5"/>
       <x:c r="B121" s="5" t="str">
-        <x:v>Title-block hyperlinks must work in exported PDFs opened in other viewers. Support selected paper size with a chosen quantity or fit option; clarify whether the quantity refers to pages or title blocks.</x:v>
+        <x:v>Title-block hyperlinks must work in exported PDFs opened in other viewers. Support selected paper size with a chosen page quantity. The previously mentioned fit option was withdrawn 2026-09-18.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1316,7 +1316,7 @@
     <x:row r="125" ht="15" hidden="0" customHeight="1">
       <x:c r="A125" s="5"/>
       <x:c r="B125" s="5" t="str">
-        <x:v>Structural break lines must expose size and placement controls, including moving the break along its segment.</x:v>
+        <x:v>Structural break lines must expose independent width, height and placement controls, including clear drag handles for each and moving the break along its segment.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="15" hidden="0" customHeight="1">
@@ -1334,7 +1334,7 @@
     <x:row r="128" ht="15" hidden="0" customHeight="1">
       <x:c r="A128" s="5"/>
       <x:c r="B128" s="5" t="str">
-        <x:v>Clarify the unfinished report “whiteout should”; retain existing Whiteout requirements pending the missing detail.</x:v>
+        <x:v>Whiteout removes only flattened PDF linework in the selected region; live editable markups must remain untouched. Scanned linework is flattened page content.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Draw PDF page tiles pixel for pixel, as sharp as a snapshot
A snapshot pasted beside its source looked sharper than the page until
zoomed in. The snapshot is drawn as vectors at the screen's resolution.
The page was drawn from tiles rendered at the next rung above the zoom
and placed at fractional pixel positions, so Qt shrank and smoothed
every tile.

Tiles are now rendered at the zoom on screen, to four significant
figures, and drawn with their corners on whole device pixels. When the
tile is its own size it is copied with no smoothing. The previous zoom's
tiles still stand in while a new zoom renders. Turned pages keep the
smoothed draw.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -488,7 +488,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="75" customHeight="1"/>
+    <row r="19" ht="75" customHeight="1">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PDF linework on the page looks blurrier than a snapshot of the same lines pasted beside it until zoomed in. Page lines must look as sharp as the pasted snapshot at every zoom.</t>
+        </is>
+      </c>
+    </row>
     <row r="20" ht="30" customHeight="1"/>
     <row r="21" ht="45" customHeight="1"/>
     <row r="22" ht="30" customHeight="1"/>

</xml_diff>

<commit_message>
Draw hatch as lines, drop the size pop-up, paint snapshots from vectors
Hatch was a tiled picture scaled by the hatch scale, so at a large scale
it was a magnified image and blurred. It is now drawn as real lines
clipped to the shape, in its own colour over the solid fill. That stays
sharp at any scale or zoom and is vector in an exported PDF.

A rectangle or ellipse still opened the exact-size dialog once placed.
The size bar while drawing is the size entry now, as in Bluebeam;
Exact size stays on the right-click menu.

A pasted snapshot showed stray repeated dots in the app but not in other
viewers. The app replayed the capture-time recording while the export
painted the kept vector source. Both now paint the vector source, cached
at screen resolution for each zoom.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -495,9 +495,27 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1"/>
-    <row r="21" ht="45" customHeight="1"/>
-    <row r="22" ht="30" customHeight="1"/>
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>A pasted snapshot shows stray repeated dots in the app that do not appear in other PDF editors. The app must draw it as the export does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>After placing a rectangle or ellipse no size dialog may pop up; the size bar while drawing is the only size entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hatch must stay sharp at any hatch scale and zoom: linework, not a tiled picture.</t>
+        </is>
+      </c>
+    </row>
     <row r="24" ht="90" customHeight="1"/>
     <row r="25" ht="45" customHeight="1"/>
     <row r="26" ht="45" customHeight="1"/>

</xml_diff>

<commit_message>
Log the 2026-09-28 decisions on the Bluebeam comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -523,15 +523,76 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="90" customHeight="1"/>
-    <row r="25" ht="45" customHeight="1"/>
-    <row r="26" ht="45" customHeight="1"/>
-    <row r="27" ht="30" customHeight="1"/>
-    <row r="28" ht="45" customHeight="1"/>
-    <row r="29" ht="30" customHeight="1"/>
-    <row r="30" ht="30" customHeight="1"/>
-    <row r="31" ht="30" customHeight="1"/>
-    <row r="32" ht="30" customHeight="1"/>
+    <row r="24" ht="90" customHeight="1">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>A1: Keep fractional font sizes exact (10.87 pt stays 10.87 pt, not rounded to a whole pixel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>A2: Draw stamp artwork (e.g. the Titleblock) as linework, not a picture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>B3: Viewports: different scales in different regions of one sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>B6: Link tool: a region that jumps to a page, a view, a file or a web address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>B8: A library of named hatches and line styles like Bluebeam's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C2: Search the PDF's own text and the markups' text across all pages, list every hit, and replace text in markups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C4: Crop pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C5: Extract or split pages into a new PDF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Markups list panel like Bluebeam's: columns for colour, line style, font and similar; filter and sort; select rows to change colour, style or delete several markups at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Panel rail buttons can move between the left and right side but cannot be reordered top to bottom by dragging. They must be.</t>
+        </is>
+      </c>
+    </row>
     <row r="36" ht="45" customHeight="1"/>
     <row r="37" ht="30" customHeight="1"/>
     <row r="38" ht="30" customHeight="1"/>

</xml_diff>

<commit_message>
Page setup panel with separate X/Y scales; viewports shown only when clicked into
A Page setup panel on the right rail follows the current page: paper size,
orientation and custom size, the scale (with an optional separate scale
down the page), units, decimal places, and the page's viewports to add,
edit or delete. Lengths, areas and rectangle sizes honour different X and
Y scales, which also travel in the PDF measurement dictionary. A viewport's
frame now shows only while it has been clicked into, or while the Viewport
tool is out. The add-leader menu uses the Callout and Cloud+ icons.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -628,10 +628,48 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="45" customHeight="1"/>
-    <row r="40" ht="30" customHeight="1"/>
-    <row r="43" ht="45" customHeight="1"/>
-    <row r="44" ht="75" customHeight="1"/>
+    <row r="39" ht="45" customHeight="1">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Add-leader menu icons must be the callout icons themselves (text box + leader + arrow for an arrow callout, text box + leader + cloud for a cloud callout), not just an arrow or just a cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A viewport's frame shows only while it has been clicked into; otherwise it is hidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Page setup and scale panel that follows the current page: units, decimal places, scale, the viewports on the page (add, change, delete), page size and orientation (e.g. landscape), and separate X and Y scales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>A Sketch Tools markup (e.g. section cut) placed in MarkForge and opened in another PDF editor does not look right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>A cloud markup opened in another editor shows a drag box of the wrong size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="75" customHeight="1">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Every markup type must export correctly to PDF and look and behave right in other editors.</t>
+        </is>
+      </c>
+    </row>
     <row r="45" ht="90" customHeight="1"/>
     <row r="46" ht="60" customHeight="1"/>
     <row r="47" ht="60" customHeight="1"/>

</xml_diff>

<commit_message>
Export and tool-set import one to one with Bluebeam; nested groups; replace image
Export: /RD written left, bottom, right, top with Rects even about the
shape, so another editor's drag box is the shape (cloud, square, circle,
callout); annotations in stacking order; borderless text says /BS /W 0;
text boxes carry /DS and /RC; colours, fill opacity, hatch, blend and
dashes as Bluebeam writes them; arcs as a curved PolyLine; groups written
as Bluebeam's /GroupNesting with nested sub-groups.

Import: nested /GroupNesting sub-groups from .btx files and Bluebeam PDFs;
/Curves, /LineStyle, hatch tiles, FreeText colours, circled text and the
callout knee; stamp artwork fitted to its box as PDF does; dash lengths in
line widths.

Images: right-click Replace image from file or clipboard, fitted into the
old picture's box keeping the new one's proportions, like Word.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -670,9 +670,27 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="90" customHeight="1"/>
-    <row r="46" ht="60" customHeight="1"/>
-    <row r="47" ht="60" customHeight="1"/>
+    <row r="45" ht="90" customHeight="1">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sketch Tools contain groups within groups. Import them as nested groups linked together the way Bluebeam does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Import of any Bluebeam tool set must be exactly one to one with Bluebeam; it currently is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Right-click an image: Replace image from clipboard or from file. The new picture keeps its own aspect ratio and is sized from the existing image, exactly like Word.</t>
+        </is>
+      </c>
+    </row>
     <row r="48" ht="45" customHeight="1"/>
     <row r="49" ht="30" customHeight="1"/>
     <row r="50" ht="90" customHeight="1"/>

</xml_diff>

<commit_message>
Every markup exports exactly as drawn, on every kind of page
Turned PDF pages: appearances carry the page's turn in their /Matrix; they
were squashed into the turned Rect. Cropped pages: display-to-file mapping
built from the crop box (MuPDF's transformation_matrix was used the wrong
way round and drops the crop on turned pages), fixing export and import.
/RD computed in file space. Turned or rounded boxes go out as their exact
outline; turned text carries /Rotation. Hatches embedded as PDF tiling
patterns. Round joins on clouds (screen drew spikes no export showed).
Freehand arrows as polylines; arrowheads filled via /IC. Notes on turned
pages upright and pinned with NoRotate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -691,7 +691,13 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="45" customHeight="1"/>
+    <row r="48" ht="45" customHeight="1">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Fix the margin bugs and every other export issue found, for every markup type throughout the app: anything added in MarkForge must appear exactly the same in another editor.</t>
+        </is>
+      </c>
+    </row>
     <row r="49" ht="30" customHeight="1"/>
     <row r="50" ht="90" customHeight="1"/>
     <row r="51" ht="30" customHeight="1"/>

</xml_diff>

<commit_message>
Bluebeam move/copy keys, page paste bar, dash spacing, format painter, viewport rescale
Move: copy only when Ctrl is held at the press; Ctrl mid-move turns
snapping off; Shift locks to lines. Measurements and sized shapes are read
again at the scale where a move or resize ends (viewport or page).
Shift/Ctrl on an outline reshapes only on a click; a drag is a constrained
move or a copy. Pages panel: Ctrl+C/Ctrl+V act on pages, with an insertion
bar under the pointer while a page is on the clipboard. Dashes kept in
points with a Spacing setting, so thickness no longer changes them; cloud
size for every cloud. Add-leader and Cloud+ pointers show the callout
drawings. Format painter carries every appearance property, stays in hand,
and paints a dragged box of markups in one step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGLSBBTU1XTPaobQaPWfi
</commit_message>
<xml_diff>
--- a/docs/tasklist.xlsx
+++ b/docs/tasklist.xlsx
@@ -350,7 +350,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -698,11 +698,55 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1"/>
-    <row r="50" ht="90" customHeight="1"/>
-    <row r="51" ht="30" customHeight="1"/>
-    <row r="54" ht="30" customHeight="1"/>
-    <row r="55" ht="30" customHeight="1"/>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Dragging a measurement into or out of a viewport changes its scale automatically: finished inside the viewport it uses the viewport's scale, otherwise the page's.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Move and copy modifiers like Bluebeam: only copy if Ctrl is held before the drag starts; during a move, Ctrl turns snapping off and Shift locks the move to straight lines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Pages panel: Ctrl+C and Ctrl+V copy and paste pages; with a page on the clipboard, hovering shows an insertion bar where it will go, exactly like Bluebeam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Cloud size property for clouds, and a spacing (scale) property for line types that scales dot and dash spacing; line thickness must not change the spacing (it currently does).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>The add-leader icons are still wrong; fix them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Adding a curve or control point with Shift+click or Ctrl+click must not happen when the item is dragged afterwards; that is a Shift-drag or Ctrl-drag instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Format painter must behave exactly like Bluebeam's.</t>
+        </is>
+      </c>
+    </row>
     <row r="57" ht="30" customHeight="1"/>
     <row r="58" ht="30" customHeight="1"/>
     <row r="59" ht="30" customHeight="1"/>

</xml_diff>